<commit_message>
Update game data: fix Canada Malmo 2026 entry and add opponent scouting data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026/public/games/Canada_FIFH_Malmo_2026.xlsx
+++ b/2026/public/games/Canada_FIFH_Malmo_2026.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb80e08bdabfb8fb/Documents/NAC SPORT DATA/Categories/Malmo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmui\Claude Projects\goalball-dashboard\2026\public\games\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_14309207ADC42E926F7E5614B9EB3C0309F20B4C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73348466-24C0-4733-AB0E-2751118EBDAC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0FBF67-1267-43BB-887A-E54D3722AA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$ZX$192</definedName>
+  </definedNames>
   <calcPr calcId="114210"/>
 </workbook>
 </file>
@@ -4045,6 +4048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:ZX192"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -6150,7 +6154,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="2" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6167,7 +6171,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="3" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -6184,7 +6188,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -6216,7 +6220,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="5" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -6248,7 +6252,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="6" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -6280,7 +6284,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="7" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
@@ -6312,7 +6316,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="8" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3</v>
       </c>
@@ -6344,7 +6348,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="9" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
@@ -6376,7 +6380,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="10" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -6408,7 +6412,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="11" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4</v>
       </c>
@@ -6440,7 +6444,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="12" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5</v>
       </c>
@@ -6472,7 +6476,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="13" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5</v>
       </c>
@@ -6504,7 +6508,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="14" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>6</v>
       </c>
@@ -6536,7 +6540,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="15" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6</v>
       </c>
@@ -6568,7 +6572,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="16" spans="1:700" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:700" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>7</v>
       </c>
@@ -6600,7 +6604,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>7</v>
       </c>
@@ -6632,7 +6636,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>8</v>
       </c>
@@ -6664,7 +6668,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>8</v>
       </c>
@@ -6696,7 +6700,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>9</v>
       </c>
@@ -6728,7 +6732,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>9</v>
       </c>
@@ -6760,7 +6764,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>10</v>
       </c>
@@ -6792,7 +6796,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>10</v>
       </c>
@@ -6824,7 +6828,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>11</v>
       </c>
@@ -6856,7 +6860,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>11</v>
       </c>
@@ -6888,7 +6892,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>12</v>
       </c>
@@ -6920,7 +6924,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>12</v>
       </c>
@@ -6952,7 +6956,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>13</v>
       </c>
@@ -6984,7 +6988,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>13</v>
       </c>
@@ -7016,7 +7020,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>14</v>
       </c>
@@ -7048,7 +7052,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>14</v>
       </c>
@@ -7080,7 +7084,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>15</v>
       </c>
@@ -7112,7 +7116,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>15</v>
       </c>
@@ -7144,7 +7148,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>16</v>
       </c>
@@ -7176,7 +7180,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>16</v>
       </c>
@@ -7208,7 +7212,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>17</v>
       </c>
@@ -7240,7 +7244,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>17</v>
       </c>
@@ -7272,7 +7276,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>18</v>
       </c>
@@ -7304,7 +7308,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>18</v>
       </c>
@@ -7336,7 +7340,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>19</v>
       </c>
@@ -7368,7 +7372,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>19</v>
       </c>
@@ -7400,7 +7404,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>20</v>
       </c>
@@ -7432,7 +7436,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>20</v>
       </c>
@@ -7464,7 +7468,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>21</v>
       </c>
@@ -7496,7 +7500,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>21</v>
       </c>
@@ -7528,7 +7532,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>22</v>
       </c>
@@ -7560,7 +7564,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>22</v>
       </c>
@@ -7592,7 +7596,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>23</v>
       </c>
@@ -7624,7 +7628,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>23</v>
       </c>
@@ -7656,7 +7660,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>24</v>
       </c>
@@ -7720,7 +7724,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>25</v>
       </c>
@@ -7752,7 +7756,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>25</v>
       </c>
@@ -7784,7 +7788,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>26</v>
       </c>
@@ -7816,7 +7820,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>26</v>
       </c>
@@ -7848,7 +7852,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>27</v>
       </c>
@@ -7912,7 +7916,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>28</v>
       </c>
@@ -7944,7 +7948,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>28</v>
       </c>
@@ -7976,7 +7980,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>29</v>
       </c>
@@ -8008,7 +8012,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>29</v>
       </c>
@@ -8040,7 +8044,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>30</v>
       </c>
@@ -8072,7 +8076,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>30</v>
       </c>
@@ -8104,7 +8108,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>31</v>
       </c>
@@ -8133,7 +8137,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>31</v>
       </c>
@@ -8162,7 +8166,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>32</v>
       </c>
@@ -8194,7 +8198,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>32</v>
       </c>
@@ -8223,7 +8227,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>33</v>
       </c>
@@ -8255,7 +8259,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>33</v>
       </c>
@@ -8287,7 +8291,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>34</v>
       </c>
@@ -8319,7 +8323,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>34</v>
       </c>
@@ -8351,7 +8355,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>35</v>
       </c>
@@ -8383,7 +8387,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>35</v>
       </c>
@@ -8415,7 +8419,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>36</v>
       </c>
@@ -8447,7 +8451,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>36</v>
       </c>
@@ -8479,7 +8483,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>37</v>
       </c>
@@ -8543,7 +8547,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>38</v>
       </c>
@@ -8575,7 +8579,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>38</v>
       </c>
@@ -8607,7 +8611,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>39</v>
       </c>
@@ -8639,7 +8643,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>39</v>
       </c>
@@ -8671,7 +8675,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>40</v>
       </c>
@@ -8703,7 +8707,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>40</v>
       </c>
@@ -8735,7 +8739,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>41</v>
       </c>
@@ -8764,7 +8768,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>41</v>
       </c>
@@ -8796,7 +8800,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>42</v>
       </c>
@@ -8828,7 +8832,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>42</v>
       </c>
@@ -8860,7 +8864,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>43</v>
       </c>
@@ -8892,7 +8896,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>43</v>
       </c>
@@ -8924,7 +8928,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>44</v>
       </c>
@@ -8956,7 +8960,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>44</v>
       </c>
@@ -8988,7 +8992,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>45</v>
       </c>
@@ -9020,7 +9024,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>45</v>
       </c>
@@ -9052,7 +9056,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>46</v>
       </c>
@@ -9116,7 +9120,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>1</v>
       </c>
@@ -9133,7 +9137,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>1</v>
       </c>
@@ -9150,7 +9154,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2</v>
       </c>
@@ -9167,7 +9171,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>47</v>
       </c>
@@ -9199,7 +9203,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>47</v>
       </c>
@@ -9231,7 +9235,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>48</v>
       </c>
@@ -9263,7 +9267,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>48</v>
       </c>
@@ -9295,7 +9299,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>49</v>
       </c>
@@ -9327,7 +9331,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>49</v>
       </c>
@@ -9359,7 +9363,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>50</v>
       </c>
@@ -9376,7 +9380,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>50</v>
       </c>
@@ -9405,7 +9409,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>51</v>
       </c>
@@ -9437,7 +9441,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>51</v>
       </c>
@@ -9469,7 +9473,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>52</v>
       </c>
@@ -9501,7 +9505,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>52</v>
       </c>
@@ -9533,7 +9537,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>53</v>
       </c>
@@ -9565,7 +9569,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>53</v>
       </c>
@@ -9597,7 +9601,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>54</v>
       </c>
@@ -9629,7 +9633,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>54</v>
       </c>
@@ -9661,7 +9665,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>55</v>
       </c>
@@ -9693,7 +9697,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>55</v>
       </c>
@@ -9725,7 +9729,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>56</v>
       </c>
@@ -9757,7 +9761,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>56</v>
       </c>
@@ -9789,7 +9793,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>57</v>
       </c>
@@ -9821,7 +9825,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>57</v>
       </c>
@@ -9850,7 +9854,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>58</v>
       </c>
@@ -9882,7 +9886,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>58</v>
       </c>
@@ -9914,7 +9918,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>59</v>
       </c>
@@ -9946,7 +9950,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>59</v>
       </c>
@@ -9978,7 +9982,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>60</v>
       </c>
@@ -10010,7 +10014,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>60</v>
       </c>
@@ -10042,7 +10046,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>61</v>
       </c>
@@ -10074,7 +10078,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>61</v>
       </c>
@@ -10103,7 +10107,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>62</v>
       </c>
@@ -10135,7 +10139,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>62</v>
       </c>
@@ -10167,7 +10171,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>63</v>
       </c>
@@ -10199,7 +10203,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>63</v>
       </c>
@@ -10231,7 +10235,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>64</v>
       </c>
@@ -10263,7 +10267,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>64</v>
       </c>
@@ -10295,7 +10299,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>65</v>
       </c>
@@ -10327,7 +10331,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>65</v>
       </c>
@@ -10359,7 +10363,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>66</v>
       </c>
@@ -10391,7 +10395,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>66</v>
       </c>
@@ -10423,7 +10427,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>67</v>
       </c>
@@ -10455,7 +10459,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>67</v>
       </c>
@@ -10490,7 +10494,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>68</v>
       </c>
@@ -10522,7 +10526,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>68</v>
       </c>
@@ -10554,7 +10558,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>69</v>
       </c>
@@ -10586,7 +10590,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>69</v>
       </c>
@@ -10618,7 +10622,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>70</v>
       </c>
@@ -10650,7 +10654,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>70</v>
       </c>
@@ -10682,7 +10686,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>71</v>
       </c>
@@ -10711,7 +10715,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>71</v>
       </c>
@@ -10740,7 +10744,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>72</v>
       </c>
@@ -10775,7 +10779,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>73</v>
       </c>
@@ -10807,7 +10811,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>72</v>
       </c>
@@ -10836,7 +10840,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>74</v>
       </c>
@@ -10868,7 +10872,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>73</v>
       </c>
@@ -10900,7 +10904,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>75</v>
       </c>
@@ -10932,7 +10936,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>74</v>
       </c>
@@ -10961,7 +10965,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>76</v>
       </c>
@@ -10990,7 +10994,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>75</v>
       </c>
@@ -11022,7 +11026,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>77</v>
       </c>
@@ -11054,7 +11058,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>76</v>
       </c>
@@ -11086,7 +11090,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>78</v>
       </c>
@@ -11118,7 +11122,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>77</v>
       </c>
@@ -11147,7 +11151,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>79</v>
       </c>
@@ -11179,7 +11183,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>78</v>
       </c>
@@ -11211,7 +11215,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>80</v>
       </c>
@@ -11243,7 +11247,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>79</v>
       </c>
@@ -11272,7 +11276,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>81</v>
       </c>
@@ -11304,7 +11308,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>80</v>
       </c>
@@ -11336,7 +11340,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>82</v>
       </c>
@@ -11368,7 +11372,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>81</v>
       </c>
@@ -11400,7 +11404,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>83</v>
       </c>
@@ -11432,7 +11436,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>82</v>
       </c>
@@ -11461,7 +11465,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>84</v>
       </c>
@@ -11493,7 +11497,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>83</v>
       </c>
@@ -11525,7 +11529,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>85</v>
       </c>
@@ -11557,7 +11561,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>84</v>
       </c>
@@ -11589,7 +11593,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>86</v>
       </c>
@@ -11621,7 +11625,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>85</v>
       </c>
@@ -11653,7 +11657,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>87</v>
       </c>
@@ -11688,7 +11692,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>88</v>
       </c>
@@ -11720,7 +11724,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>86</v>
       </c>
@@ -11752,7 +11756,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>89</v>
       </c>
@@ -11784,7 +11788,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>87</v>
       </c>
@@ -11833,7 +11837,7 @@
         <v>1204</v>
       </c>
       <c r="G183" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="H183" t="s">
         <v>716</v>
@@ -11848,7 +11852,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>88</v>
       </c>
@@ -11880,7 +11884,7 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>91</v>
       </c>
@@ -11912,7 +11916,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>89</v>
       </c>
@@ -11944,7 +11948,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>92</v>
       </c>
@@ -11976,7 +11980,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>90</v>
       </c>
@@ -12008,7 +12012,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>93</v>
       </c>
@@ -12040,7 +12044,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>91</v>
       </c>
@@ -12072,7 +12076,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>94</v>
       </c>
@@ -12104,7 +12108,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>2</v>
       </c>
@@ -12122,6 +12126,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:ZX192" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Goal Canada"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>